<commit_message>
Actualizacion automatica del tablero
</commit_message>
<xml_diff>
--- a/MATRIZ_MAESTRA_DECISIONES_Trazabilidad.xlsx
+++ b/MATRIZ_MAESTRA_DECISIONES_Trazabilidad.xlsx
@@ -1350,7 +1350,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1368,11 +1368,41 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>VERDE</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>3318</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
           <t>AMARILLO</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>1</v>
+      <c r="B3" t="n">
+        <v>1505</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ROJO</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>751</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>NEGRO</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>111</v>
       </c>
     </row>
   </sheetData>

</xml_diff>